<commit_message>
draw every grouping's Figure 1 from one walkthrough
</commit_message>
<xml_diff>
--- a/05_Figures/HRvLR/F1_Overview/c_data/f1_overview.xlsx
+++ b/05_Figures/HRvLR/F1_Overview/c_data/f1_overview.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2764" uniqueCount="407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2791" uniqueCount="422">
   <si>
     <t>sheet</t>
   </si>
@@ -784,16 +784,16 @@
     <t>contrasts</t>
   </si>
   <si>
-    <t>02_HRvLR_groups/02_Protein_Contrasts/c_data/protein_contrasts.xlsx</t>
-  </si>
-  <si>
-    <t>0d6cf853ff8d0d35c8767a6734aeecb9</t>
+    <t>03_Group_comparisons/HRvLR/02_Protein_Contrasts/c_data/protein_contrasts.xlsx</t>
+  </si>
+  <si>
+    <t>4a09b3edb7bc9a8d0cee075927563827</t>
   </si>
   <si>
     <t>set_tests</t>
   </si>
   <si>
-    <t>02_HRvLR_groups/03_Set_Contrasts/c_data/set_tests.rds</t>
+    <t>03_Group_comparisons/HRvLR/03_Set_Contrasts/c_data/set_tests.rds</t>
   </si>
   <si>
     <t>b928dfb75f0631b92e8ffaf819778f86</t>
@@ -808,7 +808,7 @@
     <t>bc1bf66e89df936e164c317354990470</t>
   </si>
   <si>
-    <t>00_Input/phenotype.csv</t>
+    <t>00_Setup/Input/phenotype.csv</t>
   </si>
   <si>
     <t>5a1989db406daa0b70189a9f0df52cf3</t>
@@ -817,7 +817,7 @@
     <t>design</t>
   </si>
   <si>
-    <t>02_HRvLR_groups/Figures/F1_Overview/assets/design.png</t>
+    <t>05_Figures/HRvLR/F1_Overview/assets/design.png</t>
   </si>
   <si>
     <t>3839c802fb7bae43324ab254e10a7a9d</t>
@@ -931,12 +931,24 @@
     <t>1.2.1</t>
   </si>
   <si>
+    <t>evaluate</t>
+  </si>
+  <si>
+    <t>1.0.5</t>
+  </si>
+  <si>
     <t>farver</t>
   </si>
   <si>
     <t>2.1.2</t>
   </si>
   <si>
+    <t>fastmap</t>
+  </si>
+  <si>
+    <t>1.2.0</t>
+  </si>
+  <si>
     <t>foreach</t>
   </si>
   <si>
@@ -1009,6 +1021,18 @@
     <t>1.1.4</t>
   </si>
   <si>
+    <t>htmltools</t>
+  </si>
+  <si>
+    <t>0.5.9</t>
+  </si>
+  <si>
+    <t>htmlwidgets</t>
+  </si>
+  <si>
+    <t>1.6.4</t>
+  </si>
+  <si>
     <t>IRanges</t>
   </si>
   <si>
@@ -1021,6 +1045,15 @@
     <t>1.0.14</t>
   </si>
   <si>
+    <t>jsonlite</t>
+  </si>
+  <si>
+    <t>knitr</t>
+  </si>
+  <si>
+    <t>1.51</t>
+  </si>
+  <si>
     <t>labeling</t>
   </si>
   <si>
@@ -1030,9 +1063,6 @@
     <t>lifecycle</t>
   </si>
   <si>
-    <t>1.0.5</t>
-  </si>
-  <si>
     <t>limma</t>
   </si>
   <si>
@@ -1069,6 +1099,9 @@
     <t>1.5.0</t>
   </si>
   <si>
+    <t>otel</t>
+  </si>
+  <si>
     <t>patchwork</t>
   </si>
   <si>
@@ -1147,6 +1180,12 @@
     <t>1.3.0</t>
   </si>
   <si>
+    <t>rmarkdown</t>
+  </si>
+  <si>
+    <t>2.31</t>
+  </si>
+  <si>
     <t>rprojroot</t>
   </si>
   <si>
@@ -1244,6 +1283,12 @@
   </si>
   <si>
     <t>xml2</t>
+  </si>
+  <si>
+    <t>yaml</t>
+  </si>
+  <si>
+    <t>2.3.12</t>
   </si>
 </sst>
 </file>
@@ -1684,7 +1729,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -1959,15 +2004,15 @@
         <v>315</v>
       </c>
       <c r="C25" t="s">
-        <v>316</v>
+        <v>271</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
+        <v>316</v>
+      </c>
+      <c r="B26" t="s">
         <v>317</v>
-      </c>
-      <c r="B26" t="s">
-        <v>307</v>
       </c>
       <c r="C26" t="s">
         <v>271</v>
@@ -1981,15 +2026,15 @@
         <v>319</v>
       </c>
       <c r="C27" t="s">
-        <v>271</v>
+        <v>320</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B28" t="s">
-        <v>321</v>
+        <v>311</v>
       </c>
       <c r="C28" t="s">
         <v>271</v>
@@ -2036,7 +2081,7 @@
         <v>329</v>
       </c>
       <c r="C32" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -2091,7 +2136,7 @@
         <v>339</v>
       </c>
       <c r="C37" t="s">
-        <v>316</v>
+        <v>271</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -2099,7 +2144,7 @@
         <v>340</v>
       </c>
       <c r="B38" t="s">
-        <v>341</v>
+        <v>291</v>
       </c>
       <c r="C38" t="s">
         <v>271</v>
@@ -2107,10 +2152,10 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
+        <v>341</v>
+      </c>
+      <c r="B39" t="s">
         <v>342</v>
-      </c>
-      <c r="B39" t="s">
-        <v>343</v>
       </c>
       <c r="C39" t="s">
         <v>271</v>
@@ -2118,10 +2163,10 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
+        <v>343</v>
+      </c>
+      <c r="B40" t="s">
         <v>344</v>
-      </c>
-      <c r="B40" t="s">
-        <v>345</v>
       </c>
       <c r="C40" t="s">
         <v>271</v>
@@ -2129,10 +2174,10 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B41" t="s">
-        <v>347</v>
+        <v>303</v>
       </c>
       <c r="C41" t="s">
         <v>271</v>
@@ -2140,32 +2185,32 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B42" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C42" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="B43" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C43" t="s">
-        <v>271</v>
+        <v>320</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="B44" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C44" t="s">
         <v>271</v>
@@ -2173,10 +2218,10 @@
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B45" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="C45" t="s">
         <v>271</v>
@@ -2184,10 +2229,10 @@
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B46" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C46" t="s">
         <v>271</v>
@@ -2195,10 +2240,10 @@
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B47" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="C47" t="s">
         <v>271</v>
@@ -2206,10 +2251,10 @@
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B48" t="s">
-        <v>361</v>
+        <v>319</v>
       </c>
       <c r="C48" t="s">
         <v>271</v>
@@ -2217,10 +2262,10 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="B49" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="C49" t="s">
         <v>271</v>
@@ -2228,10 +2273,10 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B50" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="C50" t="s">
         <v>271</v>
@@ -2239,10 +2284,10 @@
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B51" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="C51" t="s">
         <v>271</v>
@@ -2250,10 +2295,10 @@
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="B52" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="C52" t="s">
         <v>271</v>
@@ -2261,10 +2306,10 @@
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B53" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="C53" t="s">
         <v>271</v>
@@ -2272,21 +2317,21 @@
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="B54" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="C54" t="s">
-        <v>316</v>
+        <v>271</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="B55" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="C55" t="s">
         <v>271</v>
@@ -2294,21 +2339,21 @@
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="B56" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="C56" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="B57" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="C57" t="s">
         <v>271</v>
@@ -2316,10 +2361,10 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="B58" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="C58" t="s">
         <v>271</v>
@@ -2327,10 +2372,10 @@
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="B59" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="C59" t="s">
         <v>271</v>
@@ -2338,10 +2383,10 @@
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="B60" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="C60" t="s">
         <v>271</v>
@@ -2349,21 +2394,21 @@
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="B61" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="C61" t="s">
-        <v>271</v>
+        <v>320</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="B62" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="C62" t="s">
         <v>271</v>
@@ -2371,10 +2416,10 @@
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="B63" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="C63" t="s">
         <v>271</v>
@@ -2382,21 +2427,21 @@
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="B64" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="C64" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="B65" t="s">
-        <v>349</v>
+        <v>392</v>
       </c>
       <c r="C65" t="s">
         <v>271</v>
@@ -2404,10 +2449,10 @@
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="B66" t="s">
-        <v>301</v>
+        <v>394</v>
       </c>
       <c r="C66" t="s">
         <v>271</v>
@@ -2415,10 +2460,10 @@
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
+        <v>395</v>
+      </c>
+      <c r="B67" t="s">
         <v>396</v>
-      </c>
-      <c r="B67" t="s">
-        <v>397</v>
       </c>
       <c r="C67" t="s">
         <v>271</v>
@@ -2426,10 +2471,10 @@
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
+        <v>397</v>
+      </c>
+      <c r="B68" t="s">
         <v>398</v>
-      </c>
-      <c r="B68" t="s">
-        <v>399</v>
       </c>
       <c r="C68" t="s">
         <v>271</v>
@@ -2437,10 +2482,10 @@
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
+        <v>399</v>
+      </c>
+      <c r="B69" t="s">
         <v>400</v>
-      </c>
-      <c r="B69" t="s">
-        <v>401</v>
       </c>
       <c r="C69" t="s">
         <v>271</v>
@@ -2448,10 +2493,10 @@
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
+        <v>401</v>
+      </c>
+      <c r="B70" t="s">
         <v>402</v>
-      </c>
-      <c r="B70" t="s">
-        <v>403</v>
       </c>
       <c r="C70" t="s">
         <v>271</v>
@@ -2459,10 +2504,10 @@
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
+        <v>403</v>
+      </c>
+      <c r="B71" t="s">
         <v>404</v>
-      </c>
-      <c r="B71" t="s">
-        <v>405</v>
       </c>
       <c r="C71" t="s">
         <v>271</v>
@@ -2470,12 +2515,111 @@
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
+        <v>405</v>
+      </c>
+      <c r="B72" t="s">
         <v>406</v>
       </c>
-      <c r="B72" t="s">
-        <v>305</v>
-      </c>
       <c r="C72" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" t="s">
+        <v>407</v>
+      </c>
+      <c r="B73" t="s">
+        <v>360</v>
+      </c>
+      <c r="C73" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3">
+      <c r="A74" t="s">
+        <v>408</v>
+      </c>
+      <c r="B74" t="s">
+        <v>301</v>
+      </c>
+      <c r="C74" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3">
+      <c r="A75" t="s">
+        <v>409</v>
+      </c>
+      <c r="B75" t="s">
+        <v>410</v>
+      </c>
+      <c r="C75" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3">
+      <c r="A76" t="s">
+        <v>411</v>
+      </c>
+      <c r="B76" t="s">
+        <v>412</v>
+      </c>
+      <c r="C76" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3">
+      <c r="A77" t="s">
+        <v>413</v>
+      </c>
+      <c r="B77" t="s">
+        <v>414</v>
+      </c>
+      <c r="C77" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3">
+      <c r="A78" t="s">
+        <v>415</v>
+      </c>
+      <c r="B78" t="s">
+        <v>416</v>
+      </c>
+      <c r="C78" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3">
+      <c r="A79" t="s">
+        <v>417</v>
+      </c>
+      <c r="B79" t="s">
+        <v>418</v>
+      </c>
+      <c r="C79" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3">
+      <c r="A80" t="s">
+        <v>419</v>
+      </c>
+      <c r="B80" t="s">
+        <v>309</v>
+      </c>
+      <c r="C80" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3">
+      <c r="A81" t="s">
+        <v>420</v>
+      </c>
+      <c r="B81" t="s">
+        <v>421</v>
+      </c>
+      <c r="C81" t="s">
         <v>271</v>
       </c>
     </row>

</xml_diff>